<commit_message>
Kıyaslama raporu tek sayfada hiyerarşik birleştirildi (kategori+amaç)
Doruk_Butce_Kiyaslama_Raporu.xlsx yeniden düzenlendi:
- Tek sayfa '1. Kategori + Amaç Kıyaslama': her ana kategori (kalın alt
  toplam) altında amaç kırılımı; kolonlar yan yana Gerçekleşen / 60K /
  +10K(70K) / +20K(80K); aylık + günlük blok; gerçekleşene göre fark satırı
- Kategori toplamları amaç satırlarının SUM'u; ek yalnız doktor öne çıkarma
  satırına, kategori toplamına otomatik taşınır
- Ayrı Ana Kategori / Amaç / Detay sekmeleri kaldırıldı (tek sayfada birleşti)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K7hgff2BWCVCb6R8MUC7bZ
</commit_message>
<xml_diff>
--- a/meta analiz/Doruk_Butce_Kiyaslama_Raporu.xlsx
+++ b/meta analiz/Doruk_Butce_Kiyaslama_Raporu.xlsx
@@ -7,10 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="1. Ana Kategori Kıyaslama" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="2. Amaç Kıyaslama" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="3. Sayfa x Amaç Detay" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Veri" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="1. Kategori + Amaç Kıyaslama" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Veri" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,11 +17,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##0 &quot;TL&quot;"/>
-    <numFmt numFmtId="165" formatCode="+#,##0 &quot;TL&quot;;-#,##0 &quot;TL&quot;"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="+#,##0 &quot;TL&quot;;-#,##0 &quot;TL&quot;;0"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -75,25 +74,36 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="00333333"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001A1A1A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="001A1A1A"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <b val="1"/>
       <color rgb="006D4C7D"/>
-      <sz val="10"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
       <i val="1"/>
       <color rgb="002E7D32"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="006B7280"/>
       <sz val="9"/>
     </font>
     <font>
@@ -105,36 +115,7 @@
     <font>
       <name val="Arial"/>
       <i val="1"/>
-      <color rgb="006B7280"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
       <color rgb="00777777"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="001F3A5F"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="000000FF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="001A1A1A"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="006D4C7D"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -157,12 +138,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E7D8A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F5F9FB"/>
+        <fgColor rgb="00C8A45C"/>
       </patternFill>
     </fill>
     <fill>
@@ -172,12 +148,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="006D4C7D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="006B7280"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C8A45C"/>
+        <fgColor rgb="002E7D8A"/>
       </patternFill>
     </fill>
   </fills>
@@ -207,7 +188,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -215,83 +196,67 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="10" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="10" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="11" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="10" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="18" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -659,1109 +624,775 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:J28"/>
+  <dimension ref="B2:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="3" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="2" ht="26" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Ana Kategori Kıyaslama</t>
+          <t>KATEGORİ + AMAÇ KIYASLAMA (Kategori üstte · amaç altında)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Gerçekleşen (23 Haz–22 Tem 2026) ile günlük 60K bütçe ve doktor +10K/+20K senaryoları yan yana. Ek bütçe yalnızca doktor sayfalarına (=Instagram Öne Çıkarma) eklenir.</t>
+          <t>Her ana kategori (kalın) altında amaç kırılımı. Kolonlar yan yana: Gerçekleşen (23 Haz–22 Tem 2026) · Mevcut Bütçe 60K · Doktora +10K (70K) · Doktora +20K (80K). Ek bütçe yalnız doktor sayfalarına (=Instagram Öne Çıkarma) eklenir; hastane/estetik sabit.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>PARAMETRELER (sarı = değiştirilebilir)</t>
-        </is>
+          <t>PARAMETRELER →</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Bütçe 60K:</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>60000</v>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Ek A:</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>10000</v>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Mevcut günlük bütçe (TL)</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="n">
-        <v>60000</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Doktor Ek — Senaryo A (TL)</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Doktor Ek — Senaryo B (TL)</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="n">
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Ek B:</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="n">
         <v>20000</v>
       </c>
     </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>AYLIK KIYASLAMA (TL / 30 gün) — Gerçekleşen = gerçek 30 günlük tutar</t>
+        </is>
+      </c>
+    </row>
     <row r="9">
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Gün sayısı (aylık)</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>GÜNLÜK KIYASLAMA (TL / gün)  —  Gerçekleşen = 30g toplam ÷ 30</t>
-        </is>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Kategori / Amaç</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Gerçekleşen</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Pay %</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Mevcut Bütçe 60K</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Doktora +10K (70K)</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Doktora +20K (80K)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Hastane (Kurumsal)</t>
+        </is>
+      </c>
+      <c r="C10" s="10">
+        <f>SUM(C11:C13)</f>
+        <v/>
+      </c>
+      <c r="D10" s="11">
+        <f>SUM(D11:D13)</f>
+        <v/>
+      </c>
+      <c r="E10" s="10">
+        <f>SUM(E11:E13)</f>
+        <v/>
+      </c>
+      <c r="F10" s="10">
+        <f>SUM(F11:F13)</f>
+        <v/>
+      </c>
+      <c r="G10" s="10">
+        <f>SUM(G11:G13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Lead Toplama (Form)</t>
+        </is>
+      </c>
+      <c r="C11" s="13">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Lead Toplama (Form)"))/1</f>
+        <v/>
+      </c>
+      <c r="D11" s="14">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Lead Toplama (Form)"))/SUM(Veri!$D$2:$D$763)</f>
+        <v/>
+      </c>
+      <c r="E11" s="13">
+        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Lead Toplama (Form)")/SUM(Veri!$D$2:$D$763))*$D$5)*30</f>
+        <v/>
+      </c>
+      <c r="F11" s="13">
+        <f>(((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Lead Toplama (Form)")/SUM(Veri!$D$2:$D$763))*$D$5)+0)*30</f>
+        <v/>
+      </c>
+      <c r="G11" s="13">
+        <f>(((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Lead Toplama (Form)")/SUM(Veri!$D$2:$D$763))*$D$5)+0)*30</f>
+        <v/>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>Kategori</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>Instagram Öne Çıkarma</t>
+        </is>
+      </c>
+      <c r="C12" s="13">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Instagram Öne Çıkarma"))/1</f>
+        <v/>
+      </c>
+      <c r="D12" s="14">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Instagram Öne Çıkarma"))/SUM(Veri!$D$2:$D$763)</f>
+        <v/>
+      </c>
+      <c r="E12" s="13">
+        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$5)*30</f>
+        <v/>
+      </c>
+      <c r="F12" s="13">
+        <f>(((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$5)+0)*30</f>
+        <v/>
+      </c>
+      <c r="G12" s="13">
+        <f>(((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$5)+0)*30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>Marka Bilinirliği (Erişim)</t>
+        </is>
+      </c>
+      <c r="C13" s="13">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Marka Bilinirliği (Erişim)"))/1</f>
+        <v/>
+      </c>
+      <c r="D13" s="14">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Marka Bilinirliği (Erişim)"))/SUM(Veri!$D$2:$D$763)</f>
+        <v/>
+      </c>
+      <c r="E13" s="13">
+        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Marka Bilinirliği (Erişim)")/SUM(Veri!$D$2:$D$763))*$D$5)*30</f>
+        <v/>
+      </c>
+      <c r="F13" s="13">
+        <f>(((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Marka Bilinirliği (Erişim)")/SUM(Veri!$D$2:$D$763))*$D$5)+0)*30</f>
+        <v/>
+      </c>
+      <c r="G13" s="13">
+        <f>(((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Marka Bilinirliği (Erişim)")/SUM(Veri!$D$2:$D$763))*$D$5)+0)*30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>Estetik Marka</t>
+        </is>
+      </c>
+      <c r="C14" s="16">
+        <f>SUM(C15:C16)</f>
+        <v/>
+      </c>
+      <c r="D14" s="17">
+        <f>SUM(D15:D16)</f>
+        <v/>
+      </c>
+      <c r="E14" s="16">
+        <f>SUM(E15:E16)</f>
+        <v/>
+      </c>
+      <c r="F14" s="16">
+        <f>SUM(F15:F16)</f>
+        <v/>
+      </c>
+      <c r="G14" s="16">
+        <f>SUM(G15:G16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>Lead Toplama (Form)</t>
+        </is>
+      </c>
+      <c r="C15" s="13">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Lead Toplama (Form)"))/1</f>
+        <v/>
+      </c>
+      <c r="D15" s="14">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Lead Toplama (Form)"))/SUM(Veri!$D$2:$D$763)</f>
+        <v/>
+      </c>
+      <c r="E15" s="13">
+        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Lead Toplama (Form)")/SUM(Veri!$D$2:$D$763))*$D$5)*30</f>
+        <v/>
+      </c>
+      <c r="F15" s="13">
+        <f>(((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Lead Toplama (Form)")/SUM(Veri!$D$2:$D$763))*$D$5)+0)*30</f>
+        <v/>
+      </c>
+      <c r="G15" s="13">
+        <f>(((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Lead Toplama (Form)")/SUM(Veri!$D$2:$D$763))*$D$5)+0)*30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Instagram Öne Çıkarma</t>
+        </is>
+      </c>
+      <c r="C16" s="13">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Instagram Öne Çıkarma"))/1</f>
+        <v/>
+      </c>
+      <c r="D16" s="14">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Instagram Öne Çıkarma"))/SUM(Veri!$D$2:$D$763)</f>
+        <v/>
+      </c>
+      <c r="E16" s="13">
+        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$5)*30</f>
+        <v/>
+      </c>
+      <c r="F16" s="13">
+        <f>(((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$5)+0)*30</f>
+        <v/>
+      </c>
+      <c r="G16" s="13">
+        <f>(((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$5)+0)*30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>Doktor Sayfaları</t>
+        </is>
+      </c>
+      <c r="C17" s="19">
+        <f>SUM(C18:C18)</f>
+        <v/>
+      </c>
+      <c r="D17" s="20">
+        <f>SUM(D18:D18)</f>
+        <v/>
+      </c>
+      <c r="E17" s="19">
+        <f>SUM(E18:E18)</f>
+        <v/>
+      </c>
+      <c r="F17" s="19">
+        <f>SUM(F18:F18)</f>
+        <v/>
+      </c>
+      <c r="G17" s="19">
+        <f>SUM(G18:G18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="21" t="inlineStr">
+        <is>
+          <t>Instagram Öne Çıkarma</t>
+        </is>
+      </c>
+      <c r="C18" s="22">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Doktor Sayfaları",Veri!$C$2:$C$763,"Instagram Öne Çıkarma"))/1</f>
+        <v/>
+      </c>
+      <c r="D18" s="23">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Doktor Sayfaları",Veri!$C$2:$C$763,"Instagram Öne Çıkarma"))/SUM(Veri!$D$2:$D$763)</f>
+        <v/>
+      </c>
+      <c r="E18" s="22">
+        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Doktor Sayfaları",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$5)*30</f>
+        <v/>
+      </c>
+      <c r="F18" s="22">
+        <f>(((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Doktor Sayfaları",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$5)+$F$5)*30</f>
+        <v/>
+      </c>
+      <c r="G18" s="22">
+        <f>(((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Doktor Sayfaları",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$5)+$F$6)*30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="24" t="inlineStr">
+        <is>
+          <t>GENEL TOPLAM</t>
+        </is>
+      </c>
+      <c r="C19" s="25">
+        <f>C10+C14+C17</f>
+        <v/>
+      </c>
+      <c r="D19" s="26">
+        <f>D10+D14+D17</f>
+        <v/>
+      </c>
+      <c r="E19" s="25">
+        <f>E10+E14+E17</f>
+        <v/>
+      </c>
+      <c r="F19" s="25">
+        <f>F10+F14+F17</f>
+        <v/>
+      </c>
+      <c r="G19" s="25">
+        <f>G10+G14+G17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="27" t="inlineStr">
+        <is>
+          <t>Δ Senaryo − Gerçekleşen (toplam)</t>
+        </is>
+      </c>
+      <c r="C20" s="28" t="inlineStr">
+        <is>
+          <t>(baz)</t>
+        </is>
+      </c>
+      <c r="E20" s="29">
+        <f>E19-$C$19</f>
+        <v/>
+      </c>
+      <c r="F20" s="29">
+        <f>F19-$C$19</f>
+        <v/>
+      </c>
+      <c r="G20" s="29">
+        <f>G19-$C$19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="24" customHeight="1">
+      <c r="B22" s="30" t="inlineStr">
+        <is>
+          <t>GÜNLÜK KIYASLAMA (TL / gün) — Gerçekleşen = 30 günlük ÷ 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="31" t="inlineStr">
+        <is>
+          <t>Kategori / Amaç</t>
+        </is>
+      </c>
+      <c r="C23" s="31" t="inlineStr">
         <is>
           <t>Gerçekleşen</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D23" s="31" t="inlineStr">
+        <is>
+          <t>Pay %</t>
+        </is>
+      </c>
+      <c r="E23" s="31" t="inlineStr">
         <is>
           <t>Mevcut Bütçe 60K</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>Senaryo A +10K (70K)</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>Senaryo B +20K (80K)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>Hastane (Kurumsal)</t>
-        </is>
-      </c>
-      <c r="C13" s="10">
-        <f>SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)")/30</f>
+      <c r="F23" s="31" t="inlineStr">
+        <is>
+          <t>Doktora +10K (70K)</t>
+        </is>
+      </c>
+      <c r="G23" s="31" t="inlineStr">
+        <is>
+          <t>Doktora +20K (80K)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Hastane (Kurumsal)</t>
+        </is>
+      </c>
+      <c r="C24" s="10">
+        <f>SUM(C25:C27)</f>
         <v/>
       </c>
-      <c r="D13" s="10">
-        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)")/SUM(Veri!$D$2:$D$763))*$D$6</f>
+      <c r="D24" s="11">
+        <f>SUM(D25:D27)</f>
         <v/>
       </c>
-      <c r="E13" s="10">
-        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)")/SUM(Veri!$D$2:$D$763))*$D$6+0</f>
+      <c r="E24" s="10">
+        <f>SUM(E25:E27)</f>
         <v/>
       </c>
-      <c r="F13" s="10">
-        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)")/SUM(Veri!$D$2:$D$763))*$D$6+0</f>
+      <c r="F24" s="10">
+        <f>SUM(F25:F27)</f>
         <v/>
       </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="11" t="inlineStr">
+      <c r="G24" s="10">
+        <f>SUM(G25:G27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>Lead Toplama (Form)</t>
+        </is>
+      </c>
+      <c r="C25" s="13">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Lead Toplama (Form)"))/30</f>
+        <v/>
+      </c>
+      <c r="D25" s="14">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Lead Toplama (Form)"))/SUM(Veri!$D$2:$D$763)</f>
+        <v/>
+      </c>
+      <c r="E25" s="13">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Lead Toplama (Form)")/SUM(Veri!$D$2:$D$763))*$D$5</f>
+        <v/>
+      </c>
+      <c r="F25" s="13">
+        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Lead Toplama (Form)")/SUM(Veri!$D$2:$D$763))*$D$5)+0</f>
+        <v/>
+      </c>
+      <c r="G25" s="13">
+        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Lead Toplama (Form)")/SUM(Veri!$D$2:$D$763))*$D$5)+0</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>Instagram Öne Çıkarma</t>
+        </is>
+      </c>
+      <c r="C26" s="13">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Instagram Öne Çıkarma"))/30</f>
+        <v/>
+      </c>
+      <c r="D26" s="14">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Instagram Öne Çıkarma"))/SUM(Veri!$D$2:$D$763)</f>
+        <v/>
+      </c>
+      <c r="E26" s="13">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$5</f>
+        <v/>
+      </c>
+      <c r="F26" s="13">
+        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$5)+0</f>
+        <v/>
+      </c>
+      <c r="G26" s="13">
+        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$5)+0</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>Marka Bilinirliği (Erişim)</t>
+        </is>
+      </c>
+      <c r="C27" s="13">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Marka Bilinirliği (Erişim)"))/30</f>
+        <v/>
+      </c>
+      <c r="D27" s="14">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Marka Bilinirliği (Erişim)"))/SUM(Veri!$D$2:$D$763)</f>
+        <v/>
+      </c>
+      <c r="E27" s="13">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Marka Bilinirliği (Erişim)")/SUM(Veri!$D$2:$D$763))*$D$5</f>
+        <v/>
+      </c>
+      <c r="F27" s="13">
+        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Marka Bilinirliği (Erişim)")/SUM(Veri!$D$2:$D$763))*$D$5)+0</f>
+        <v/>
+      </c>
+      <c r="G27" s="13">
+        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Marka Bilinirliği (Erişim)")/SUM(Veri!$D$2:$D$763))*$D$5)+0</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="15" t="inlineStr">
         <is>
           <t>Estetik Marka</t>
         </is>
       </c>
-      <c r="C14" s="12">
-        <f>SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka")/30</f>
+      <c r="C28" s="16">
+        <f>SUM(C29:C30)</f>
         <v/>
       </c>
-      <c r="D14" s="12">
-        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka")/SUM(Veri!$D$2:$D$763))*$D$6</f>
+      <c r="D28" s="17">
+        <f>SUM(D29:D30)</f>
         <v/>
       </c>
-      <c r="E14" s="12">
-        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka")/SUM(Veri!$D$2:$D$763))*$D$6+0</f>
+      <c r="E28" s="16">
+        <f>SUM(E29:E30)</f>
         <v/>
       </c>
-      <c r="F14" s="12">
-        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka")/SUM(Veri!$D$2:$D$763))*$D$6+0</f>
+      <c r="F28" s="16">
+        <f>SUM(F29:F30)</f>
         <v/>
       </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="13" t="inlineStr">
+      <c r="G28" s="16">
+        <f>SUM(G29:G30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>Lead Toplama (Form)</t>
+        </is>
+      </c>
+      <c r="C29" s="13">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Lead Toplama (Form)"))/30</f>
+        <v/>
+      </c>
+      <c r="D29" s="14">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Lead Toplama (Form)"))/SUM(Veri!$D$2:$D$763)</f>
+        <v/>
+      </c>
+      <c r="E29" s="13">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Lead Toplama (Form)")/SUM(Veri!$D$2:$D$763))*$D$5</f>
+        <v/>
+      </c>
+      <c r="F29" s="13">
+        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Lead Toplama (Form)")/SUM(Veri!$D$2:$D$763))*$D$5)+0</f>
+        <v/>
+      </c>
+      <c r="G29" s="13">
+        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Lead Toplama (Form)")/SUM(Veri!$D$2:$D$763))*$D$5)+0</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>Instagram Öne Çıkarma</t>
+        </is>
+      </c>
+      <c r="C30" s="13">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Instagram Öne Çıkarma"))/30</f>
+        <v/>
+      </c>
+      <c r="D30" s="14">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Instagram Öne Çıkarma"))/SUM(Veri!$D$2:$D$763)</f>
+        <v/>
+      </c>
+      <c r="E30" s="13">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$5</f>
+        <v/>
+      </c>
+      <c r="F30" s="13">
+        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$5)+0</f>
+        <v/>
+      </c>
+      <c r="G30" s="13">
+        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$5)+0</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="18" t="inlineStr">
         <is>
           <t>Doktor Sayfaları</t>
         </is>
       </c>
-      <c r="C15" s="14">
-        <f>SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Doktor Sayfaları")/30</f>
+      <c r="C31" s="19">
+        <f>SUM(C32:C32)</f>
         <v/>
       </c>
-      <c r="D15" s="14">
-        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Doktor Sayfaları")/SUM(Veri!$D$2:$D$763))*$D$6</f>
+      <c r="D31" s="20">
+        <f>SUM(D32:D32)</f>
         <v/>
       </c>
-      <c r="E15" s="14">
-        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Doktor Sayfaları")/SUM(Veri!$D$2:$D$763))*$D$6+$D$7</f>
+      <c r="E31" s="19">
+        <f>SUM(E32:E32)</f>
         <v/>
       </c>
-      <c r="F15" s="14">
-        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Doktor Sayfaları")/SUM(Veri!$D$2:$D$763))*$D$6+$D$8</f>
+      <c r="F31" s="19">
+        <f>SUM(F32:F32)</f>
         <v/>
       </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="15" t="inlineStr">
-        <is>
-          <t>TOPLAM</t>
-        </is>
-      </c>
-      <c r="C16" s="16">
-        <f>SUM(C13:C15)</f>
+      <c r="G31" s="19">
+        <f>SUM(G32:G32)</f>
         <v/>
       </c>
-      <c r="D16" s="16">
-        <f>SUM(D13:D15)</f>
+    </row>
+    <row r="32">
+      <c r="B32" s="21" t="inlineStr">
+        <is>
+          <t>Instagram Öne Çıkarma</t>
+        </is>
+      </c>
+      <c r="C32" s="22">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Doktor Sayfaları",Veri!$C$2:$C$763,"Instagram Öne Çıkarma"))/30</f>
         <v/>
       </c>
-      <c r="E16" s="16">
-        <f>SUM(E13:E15)</f>
+      <c r="D32" s="23">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Doktor Sayfaları",Veri!$C$2:$C$763,"Instagram Öne Çıkarma"))/SUM(Veri!$D$2:$D$763)</f>
         <v/>
       </c>
-      <c r="F16" s="16">
-        <f>SUM(F13:F15)</f>
+      <c r="E32" s="22">
+        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Doktor Sayfaları",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$5</f>
         <v/>
       </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="17" t="inlineStr">
-        <is>
-          <t>Δ Gerçekleşene göre</t>
-        </is>
-      </c>
-      <c r="C17" s="18" t="inlineStr">
+      <c r="F32" s="22">
+        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Doktor Sayfaları",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$5)+$F$5</f>
+        <v/>
+      </c>
+      <c r="G32" s="22">
+        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Doktor Sayfaları",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$5)+$F$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="24" t="inlineStr">
+        <is>
+          <t>GENEL TOPLAM</t>
+        </is>
+      </c>
+      <c r="C33" s="25">
+        <f>C24+C28+C31</f>
+        <v/>
+      </c>
+      <c r="D33" s="26">
+        <f>D24+D28+D31</f>
+        <v/>
+      </c>
+      <c r="E33" s="25">
+        <f>E24+E28+E31</f>
+        <v/>
+      </c>
+      <c r="F33" s="25">
+        <f>F24+F28+F31</f>
+        <v/>
+      </c>
+      <c r="G33" s="25">
+        <f>G24+G28+G31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="27" t="inlineStr">
+        <is>
+          <t>Δ Senaryo − Gerçekleşen (toplam)</t>
+        </is>
+      </c>
+      <c r="C34" s="28" t="inlineStr">
         <is>
           <t>(baz)</t>
         </is>
       </c>
-      <c r="D17" s="19">
-        <f>D16-$C$16</f>
+      <c r="E34" s="29">
+        <f>E33-$C$33</f>
         <v/>
       </c>
-      <c r="E17" s="19">
-        <f>E16-$C$16</f>
+      <c r="F34" s="29">
+        <f>F33-$C$33</f>
         <v/>
       </c>
-      <c r="F17" s="19">
-        <f>F16-$C$16</f>
+      <c r="G34" s="29">
+        <f>G33-$C$33</f>
         <v/>
       </c>
     </row>
-    <row r="19" ht="24" customHeight="1">
-      <c r="B19" s="20" t="inlineStr">
-        <is>
-          <t>AYLIK KIYASLAMA (TL / 30 gün)  —  Gerçekleşen = gerçek 30 günlük tutar</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="21" t="inlineStr">
-        <is>
-          <t>Kategori</t>
-        </is>
-      </c>
-      <c r="C20" s="21" t="inlineStr">
-        <is>
-          <t>Gerçekleşen</t>
-        </is>
-      </c>
-      <c r="D20" s="21" t="inlineStr">
-        <is>
-          <t>Mevcut Bütçe 60K</t>
-        </is>
-      </c>
-      <c r="E20" s="21" t="inlineStr">
-        <is>
-          <t>Senaryo A +10K (70K)</t>
-        </is>
-      </c>
-      <c r="F20" s="21" t="inlineStr">
-        <is>
-          <t>Senaryo B +20K (80K)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>Hastane (Kurumsal)</t>
-        </is>
-      </c>
-      <c r="C21" s="10">
-        <f>SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)")</f>
-        <v/>
-      </c>
-      <c r="D21" s="10">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)")/SUM(Veri!$D$2:$D$763))*$D$6)*$D$9</f>
-        <v/>
-      </c>
-      <c r="E21" s="10">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)")/SUM(Veri!$D$2:$D$763))*$D$6+0)*$D$9</f>
-        <v/>
-      </c>
-      <c r="F21" s="10">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)")/SUM(Veri!$D$2:$D$763))*$D$6+0)*$D$9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>Estetik Marka</t>
-        </is>
-      </c>
-      <c r="C22" s="12">
-        <f>SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka")</f>
-        <v/>
-      </c>
-      <c r="D22" s="12">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka")/SUM(Veri!$D$2:$D$763))*$D$6)*$D$9</f>
-        <v/>
-      </c>
-      <c r="E22" s="12">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka")/SUM(Veri!$D$2:$D$763))*$D$6+0)*$D$9</f>
-        <v/>
-      </c>
-      <c r="F22" s="12">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka")/SUM(Veri!$D$2:$D$763))*$D$6+0)*$D$9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="13" t="inlineStr">
-        <is>
-          <t>Doktor Sayfaları</t>
-        </is>
-      </c>
-      <c r="C23" s="14">
-        <f>SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Doktor Sayfaları")</f>
-        <v/>
-      </c>
-      <c r="D23" s="14">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Doktor Sayfaları")/SUM(Veri!$D$2:$D$763))*$D$6)*$D$9</f>
-        <v/>
-      </c>
-      <c r="E23" s="14">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Doktor Sayfaları")/SUM(Veri!$D$2:$D$763))*$D$6+$D$7)*$D$9</f>
-        <v/>
-      </c>
-      <c r="F23" s="14">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Doktor Sayfaları")/SUM(Veri!$D$2:$D$763))*$D$6+$D$8)*$D$9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="15" t="inlineStr">
-        <is>
-          <t>TOPLAM</t>
-        </is>
-      </c>
-      <c r="C24" s="16">
-        <f>SUM(C21:C23)</f>
-        <v/>
-      </c>
-      <c r="D24" s="16">
-        <f>SUM(D21:D23)</f>
-        <v/>
-      </c>
-      <c r="E24" s="16">
-        <f>SUM(E21:E23)</f>
-        <v/>
-      </c>
-      <c r="F24" s="16">
-        <f>SUM(F21:F23)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="17" t="inlineStr">
-        <is>
-          <t>Δ Gerçekleşene göre</t>
-        </is>
-      </c>
-      <c r="C25" s="18" t="inlineStr">
-        <is>
-          <t>(baz)</t>
-        </is>
-      </c>
-      <c r="D25" s="19">
-        <f>D24-$C$24</f>
-        <v/>
-      </c>
-      <c r="E25" s="19">
-        <f>E24-$C$24</f>
-        <v/>
-      </c>
-      <c r="F25" s="19">
-        <f>F24-$C$24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="22" t="inlineStr">
-        <is>
-          <t>Not: "Gerçekleşen" gerçek harcamadır (30 günlük). Mevcut bütçe ve senaryolar geçmiş oranlar korunarak hesaplanır; ek bütçe yalnız doktora eklenir, hastane/estetik sabit kalır.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="22" t="inlineStr">
-        <is>
-          <t>Gerçekleşen günlük ortalama aktif güne (26 gün) göre bakılırsa: toplam ≈ 38.921 TL/gün (30 günlük pencerede 4 gün yayın yoktu).</t>
+    <row r="36">
+      <c r="B36" s="32" t="inlineStr">
+        <is>
+          <t>Not: "Gerçekleşen" gerçek harcamadır. Mevcut bütçe ve senaryolar geçmiş oranlar korunarak hesaplanır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="32" t="inlineStr">
+        <is>
+          <t>Doktor sayfaları %100 Instagram Öne Çıkarma olduğundan +10K/+20K yalnız o satıra yansır; kategori toplamına otomatik taşınır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="32" t="inlineStr">
+        <is>
+          <t>Aktif gün (26) bazlı gerçekleşen günlük ortalama ≈ 38.921 TL/gün (30 günlük pencerede 4 gün yayın yoktu).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="32" t="inlineStr">
+        <is>
+          <t>Sarı hücreleri (bütçe / Ek A / Ek B) değiştirerek kendi senaryolarınızı üretebilirsiniz.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B3:J3"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="B19:F19"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B27:F27"/>
+  <mergeCells count="8">
+    <mergeCell ref="B3:G3"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B38:G38"/>
+    <mergeCell ref="B36:G36"/>
+    <mergeCell ref="B22:G22"/>
+    <mergeCell ref="B37:G37"/>
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="B39:G39"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="B2:J27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="3" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="2" ht="26" customHeight="1">
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>Amaç Kıyaslama</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Gerçekleşen (23 Haz–22 Tem 2026) ile günlük 60K bütçe ve doktor +10K/+20K senaryoları yan yana. Ek bütçe yalnızca doktor sayfalarına (=Instagram Öne Çıkarma) eklenir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>PARAMETRELER (sarı = değiştirilebilir)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Mevcut günlük bütçe (TL)</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="n">
-        <v>60000</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Doktor Ek — Senaryo A (TL)</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Doktor Ek — Senaryo B (TL)</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="n">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Gün sayısı (aylık)</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>GÜNLÜK KIYASLAMA (TL / gün)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>Kategori</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>Gerçekleşen</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>Mevcut Bütçe 60K</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>Senaryo A +10K (70K)</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>Senaryo B +20K (80K)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>Lead Toplama (Form)</t>
-        </is>
-      </c>
-      <c r="C13" s="10">
-        <f>SUMIFS(Veri!$D$2:$D$763,Veri!$C$2:$C$763,"Lead Toplama (Form)")/30</f>
-        <v/>
-      </c>
-      <c r="D13" s="10">
-        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$C$2:$C$763,"Lead Toplama (Form)")/SUM(Veri!$D$2:$D$763))*$D$6</f>
-        <v/>
-      </c>
-      <c r="E13" s="10">
-        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$C$2:$C$763,"Lead Toplama (Form)")/SUM(Veri!$D$2:$D$763))*$D$6+0</f>
-        <v/>
-      </c>
-      <c r="F13" s="10">
-        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$C$2:$C$763,"Lead Toplama (Form)")/SUM(Veri!$D$2:$D$763))*$D$6+0</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="13" t="inlineStr">
-        <is>
-          <t>Instagram Öne Çıkarma</t>
-        </is>
-      </c>
-      <c r="C14" s="14">
-        <f>SUMIFS(Veri!$D$2:$D$763,Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/30</f>
-        <v/>
-      </c>
-      <c r="D14" s="14">
-        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$6</f>
-        <v/>
-      </c>
-      <c r="E14" s="14">
-        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$6+$D$7</f>
-        <v/>
-      </c>
-      <c r="F14" s="14">
-        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$6+$D$8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>Marka Bilinirliği (Erişim)</t>
-        </is>
-      </c>
-      <c r="C15" s="10">
-        <f>SUMIFS(Veri!$D$2:$D$763,Veri!$C$2:$C$763,"Marka Bilinirliği (Erişim)")/30</f>
-        <v/>
-      </c>
-      <c r="D15" s="10">
-        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$C$2:$C$763,"Marka Bilinirliği (Erişim)")/SUM(Veri!$D$2:$D$763))*$D$6</f>
-        <v/>
-      </c>
-      <c r="E15" s="10">
-        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$C$2:$C$763,"Marka Bilinirliği (Erişim)")/SUM(Veri!$D$2:$D$763))*$D$6+0</f>
-        <v/>
-      </c>
-      <c r="F15" s="10">
-        <f>(SUMIFS(Veri!$D$2:$D$763,Veri!$C$2:$C$763,"Marka Bilinirliği (Erişim)")/SUM(Veri!$D$2:$D$763))*$D$6+0</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="15" t="inlineStr">
-        <is>
-          <t>TOPLAM</t>
-        </is>
-      </c>
-      <c r="C16" s="16">
-        <f>SUM(C13:C15)</f>
-        <v/>
-      </c>
-      <c r="D16" s="16">
-        <f>SUM(D13:D15)</f>
-        <v/>
-      </c>
-      <c r="E16" s="16">
-        <f>SUM(E13:E15)</f>
-        <v/>
-      </c>
-      <c r="F16" s="16">
-        <f>SUM(F13:F15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="17" t="inlineStr">
-        <is>
-          <t>Δ Gerçekleşene göre</t>
-        </is>
-      </c>
-      <c r="C17" s="18" t="inlineStr">
-        <is>
-          <t>(baz)</t>
-        </is>
-      </c>
-      <c r="D17" s="19">
-        <f>D16-$C$16</f>
-        <v/>
-      </c>
-      <c r="E17" s="19">
-        <f>E16-$C$16</f>
-        <v/>
-      </c>
-      <c r="F17" s="19">
-        <f>F16-$C$16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" ht="24" customHeight="1">
-      <c r="B19" s="20" t="inlineStr">
-        <is>
-          <t>AYLIK KIYASLAMA (TL / 30 gün)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="21" t="inlineStr">
-        <is>
-          <t>Kategori</t>
-        </is>
-      </c>
-      <c r="C20" s="21" t="inlineStr">
-        <is>
-          <t>Gerçekleşen</t>
-        </is>
-      </c>
-      <c r="D20" s="21" t="inlineStr">
-        <is>
-          <t>Mevcut Bütçe 60K</t>
-        </is>
-      </c>
-      <c r="E20" s="21" t="inlineStr">
-        <is>
-          <t>Senaryo A +10K (70K)</t>
-        </is>
-      </c>
-      <c r="F20" s="21" t="inlineStr">
-        <is>
-          <t>Senaryo B +20K (80K)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>Lead Toplama (Form)</t>
-        </is>
-      </c>
-      <c r="C21" s="10">
-        <f>SUMIFS(Veri!$D$2:$D$763,Veri!$C$2:$C$763,"Lead Toplama (Form)")</f>
-        <v/>
-      </c>
-      <c r="D21" s="10">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$C$2:$C$763,"Lead Toplama (Form)")/SUM(Veri!$D$2:$D$763))*$D$6)*$D$9</f>
-        <v/>
-      </c>
-      <c r="E21" s="10">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$C$2:$C$763,"Lead Toplama (Form)")/SUM(Veri!$D$2:$D$763))*$D$6+0)*$D$9</f>
-        <v/>
-      </c>
-      <c r="F21" s="10">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$C$2:$C$763,"Lead Toplama (Form)")/SUM(Veri!$D$2:$D$763))*$D$6+0)*$D$9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="13" t="inlineStr">
-        <is>
-          <t>Instagram Öne Çıkarma</t>
-        </is>
-      </c>
-      <c r="C22" s="14">
-        <f>SUMIFS(Veri!$D$2:$D$763,Veri!$C$2:$C$763,"Instagram Öne Çıkarma")</f>
-        <v/>
-      </c>
-      <c r="D22" s="14">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$6)*$D$9</f>
-        <v/>
-      </c>
-      <c r="E22" s="14">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$6+$D$7)*$D$9</f>
-        <v/>
-      </c>
-      <c r="F22" s="14">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$6+$D$8)*$D$9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>Marka Bilinirliği (Erişim)</t>
-        </is>
-      </c>
-      <c r="C23" s="10">
-        <f>SUMIFS(Veri!$D$2:$D$763,Veri!$C$2:$C$763,"Marka Bilinirliği (Erişim)")</f>
-        <v/>
-      </c>
-      <c r="D23" s="10">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$C$2:$C$763,"Marka Bilinirliği (Erişim)")/SUM(Veri!$D$2:$D$763))*$D$6)*$D$9</f>
-        <v/>
-      </c>
-      <c r="E23" s="10">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$C$2:$C$763,"Marka Bilinirliği (Erişim)")/SUM(Veri!$D$2:$D$763))*$D$6+0)*$D$9</f>
-        <v/>
-      </c>
-      <c r="F23" s="10">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$C$2:$C$763,"Marka Bilinirliği (Erişim)")/SUM(Veri!$D$2:$D$763))*$D$6+0)*$D$9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="15" t="inlineStr">
-        <is>
-          <t>TOPLAM</t>
-        </is>
-      </c>
-      <c r="C24" s="16">
-        <f>SUM(C21:C23)</f>
-        <v/>
-      </c>
-      <c r="D24" s="16">
-        <f>SUM(D21:D23)</f>
-        <v/>
-      </c>
-      <c r="E24" s="16">
-        <f>SUM(E21:E23)</f>
-        <v/>
-      </c>
-      <c r="F24" s="16">
-        <f>SUM(F21:F23)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="17" t="inlineStr">
-        <is>
-          <t>Δ Gerçekleşene göre</t>
-        </is>
-      </c>
-      <c r="C25" s="18" t="inlineStr">
-        <is>
-          <t>(baz)</t>
-        </is>
-      </c>
-      <c r="D25" s="19">
-        <f>D24-$C$24</f>
-        <v/>
-      </c>
-      <c r="E25" s="19">
-        <f>E24-$C$24</f>
-        <v/>
-      </c>
-      <c r="F25" s="19">
-        <f>F24-$C$24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="22" t="inlineStr">
-        <is>
-          <t>Not: Doktor sayfaları %100 "Instagram Öne Çıkarma" olduğundan, +10K/+20K ek bütçe bu satıra yansır. Lead ve Bilinirlik üç senaryoda da sabittir.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B3:J3"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B19:F19"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B27:F27"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="B2:G15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="2" ht="24" customHeight="1">
-      <c r="B2" s="23" t="inlineStr">
-        <is>
-          <t>Sayfa Kategorisi × Amaç — Aylık Kıyaslama (30 gün)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Her satır gerçekleşen 30g tutar ile 60K / 70K / 80K senaryolarının aylık karşılığı. Ek yalnız (Doktor Sayfaları × Instagram Öne Çıkarma) satırına eklenir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="24" t="inlineStr">
-        <is>
-          <t>Mevcut günlük bütçe →</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>60000</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="24" t="inlineStr">
-        <is>
-          <t>Doktor Ek A / B (TL) →</t>
-        </is>
-      </c>
-      <c r="D6" s="25" t="n">
-        <v>10000</v>
-      </c>
-      <c r="E6" s="25" t="n">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="26" t="inlineStr">
-        <is>
-          <t>Sayfa Kategorisi</t>
-        </is>
-      </c>
-      <c r="C8" s="26" t="inlineStr">
-        <is>
-          <t>Amaç</t>
-        </is>
-      </c>
-      <c r="D8" s="26" t="inlineStr">
-        <is>
-          <t>Gerçekleşen (30g)</t>
-        </is>
-      </c>
-      <c r="E8" s="26" t="inlineStr">
-        <is>
-          <t>60K (aylık)</t>
-        </is>
-      </c>
-      <c r="F8" s="26" t="inlineStr">
-        <is>
-          <t>+10K → 70K</t>
-        </is>
-      </c>
-      <c r="G8" s="26" t="inlineStr">
-        <is>
-          <t>+20K → 80K</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="27" t="inlineStr">
-        <is>
-          <t>Hastane (Kurumsal)</t>
-        </is>
-      </c>
-      <c r="C9" s="27" t="inlineStr">
-        <is>
-          <t>Lead Toplama (Form)</t>
-        </is>
-      </c>
-      <c r="D9" s="28">
-        <f>SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Lead Toplama (Form)")</f>
-        <v/>
-      </c>
-      <c r="E9" s="28">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Lead Toplama (Form)")/SUM(Veri!$D$2:$D$763))*$D$5)*30</f>
-        <v/>
-      </c>
-      <c r="F9" s="28">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Lead Toplama (Form)")/SUM(Veri!$D$2:$D$763))*$D$5)*30</f>
-        <v/>
-      </c>
-      <c r="G9" s="28">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Lead Toplama (Form)")/SUM(Veri!$D$2:$D$763))*$D$5)*30</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="29" t="inlineStr">
-        <is>
-          <t>Hastane (Kurumsal)</t>
-        </is>
-      </c>
-      <c r="C10" s="29" t="inlineStr">
-        <is>
-          <t>Instagram Öne Çıkarma</t>
-        </is>
-      </c>
-      <c r="D10" s="30">
-        <f>SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")</f>
-        <v/>
-      </c>
-      <c r="E10" s="30">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$5)*30</f>
-        <v/>
-      </c>
-      <c r="F10" s="30">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$5)*30</f>
-        <v/>
-      </c>
-      <c r="G10" s="30">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$5)*30</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="27" t="inlineStr">
-        <is>
-          <t>Hastane (Kurumsal)</t>
-        </is>
-      </c>
-      <c r="C11" s="27" t="inlineStr">
-        <is>
-          <t>Marka Bilinirliği (Erişim)</t>
-        </is>
-      </c>
-      <c r="D11" s="28">
-        <f>SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Marka Bilinirliği (Erişim)")</f>
-        <v/>
-      </c>
-      <c r="E11" s="28">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Marka Bilinirliği (Erişim)")/SUM(Veri!$D$2:$D$763))*$D$5)*30</f>
-        <v/>
-      </c>
-      <c r="F11" s="28">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Marka Bilinirliği (Erişim)")/SUM(Veri!$D$2:$D$763))*$D$5)*30</f>
-        <v/>
-      </c>
-      <c r="G11" s="28">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Hastane (Kurumsal)",Veri!$C$2:$C$763,"Marka Bilinirliği (Erişim)")/SUM(Veri!$D$2:$D$763))*$D$5)*30</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="29" t="inlineStr">
-        <is>
-          <t>Estetik Marka</t>
-        </is>
-      </c>
-      <c r="C12" s="29" t="inlineStr">
-        <is>
-          <t>Lead Toplama (Form)</t>
-        </is>
-      </c>
-      <c r="D12" s="30">
-        <f>SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Lead Toplama (Form)")</f>
-        <v/>
-      </c>
-      <c r="E12" s="30">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Lead Toplama (Form)")/SUM(Veri!$D$2:$D$763))*$D$5)*30</f>
-        <v/>
-      </c>
-      <c r="F12" s="30">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Lead Toplama (Form)")/SUM(Veri!$D$2:$D$763))*$D$5)*30</f>
-        <v/>
-      </c>
-      <c r="G12" s="30">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Lead Toplama (Form)")/SUM(Veri!$D$2:$D$763))*$D$5)*30</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="27" t="inlineStr">
-        <is>
-          <t>Estetik Marka</t>
-        </is>
-      </c>
-      <c r="C13" s="27" t="inlineStr">
-        <is>
-          <t>Instagram Öne Çıkarma</t>
-        </is>
-      </c>
-      <c r="D13" s="28">
-        <f>SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")</f>
-        <v/>
-      </c>
-      <c r="E13" s="28">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$5)*30</f>
-        <v/>
-      </c>
-      <c r="F13" s="28">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$5)*30</f>
-        <v/>
-      </c>
-      <c r="G13" s="28">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Estetik Marka",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$5)*30</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="31" t="inlineStr">
-        <is>
-          <t>Doktor Sayfaları</t>
-        </is>
-      </c>
-      <c r="C14" s="32" t="inlineStr">
-        <is>
-          <t>Instagram Öne Çıkarma</t>
-        </is>
-      </c>
-      <c r="D14" s="33">
-        <f>SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Doktor Sayfaları",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")</f>
-        <v/>
-      </c>
-      <c r="E14" s="33">
-        <f>((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Doktor Sayfaları",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$5)*30</f>
-        <v/>
-      </c>
-      <c r="F14" s="34">
-        <f>(((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Doktor Sayfaları",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$5)+$D$6)*30</f>
-        <v/>
-      </c>
-      <c r="G14" s="34">
-        <f>(((SUMIFS(Veri!$D$2:$D$763,Veri!$B$2:$B$763,"Doktor Sayfaları",Veri!$C$2:$C$763,"Instagram Öne Çıkarma")/SUM(Veri!$D$2:$D$763))*$D$5)+$E$6)*30</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="35" t="n"/>
-      <c r="C15" s="36" t="inlineStr">
-        <is>
-          <t>TOPLAM</t>
-        </is>
-      </c>
-      <c r="D15" s="16">
-        <f>SUM(D9:D14)</f>
-        <v/>
-      </c>
-      <c r="E15" s="16">
-        <f>SUM(E9:E14)</f>
-        <v/>
-      </c>
-      <c r="F15" s="16">
-        <f>SUM(F9:F14)</f>
-        <v/>
-      </c>
-      <c r="G15" s="16">
-        <f>SUM(G9:G14)</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="B3:G3"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B5:C5"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1777,22 +1408,22 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="37" t="inlineStr">
+      <c r="A1" s="33" t="inlineStr">
         <is>
           <t>sayfa</t>
         </is>
       </c>
-      <c r="B1" s="37" t="inlineStr">
+      <c r="B1" s="33" t="inlineStr">
         <is>
           <t>ana</t>
         </is>
       </c>
-      <c r="C1" s="37" t="inlineStr">
+      <c r="C1" s="33" t="inlineStr">
         <is>
           <t>amac</t>
         </is>
       </c>
-      <c r="D1" s="37" t="inlineStr">
+      <c r="D1" s="33" t="inlineStr">
         <is>
           <t>harcama</t>
         </is>

</xml_diff>